<commit_message>
Corporate accountability pass (batch 7) folded: 245 cases, 222 decisions
Lafarge cassation cluster (7 Sept 2021 joined arrêt — corporate CAH
complicity landmark — added to lafarge-syria), plus four new US
corporate cases with official opinion texts: Doe v. Unocal, Presbyterian
Church of Sudan v. Talisman, Doe v. Nestlé/Cargill (incl. SCOTUS 2021),
and In re Chiquita Brands (MDL line behind the June 2024 jury verdict).
Adds the BHRRC Corporate Legal Accountability lawsuit-profiles database
as a cross-reference on all corporate-defendant cases and in the README.
Coverage notes: LDH indexes no French lower courts (cours d'appel,
tribunaux correctionnels, assises) — trial-level French texts must come
from FIDH/ECCHR/TRIAL dossiers; CNDA art. 1F vein flagged for follow-up.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018QwoGBgyNDPYtcpE52gDaf
</commit_message>
<xml_diff>
--- a/international-crimes-before-courts/international-crimes-before-courts-data-v2.xlsx
+++ b/international-crimes-before-courts/international-crimes-before-courts-data-v2.xlsx
@@ -443,12 +443,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Enrichment fold</t>
+          <t>Enrichment folds</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-06 (confirmed entries from enrichment/ batches 1-5)</t>
+          <t>2026-07-06 (batches 1-5 + batch 7 corporate)</t>
         </is>
       </c>
     </row>
@@ -476,11 +476,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>National &amp; hybrid prosecutions of international crimes (main corpus, enriched)</t>
+          <t>National &amp; hybrid prosecutions (enriched)</t>
         </is>
       </c>
     </row>
@@ -491,11 +491,11 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Individual court decisions nested under each case (enriched)</t>
+          <t>Decisions nested under each case (enriched)</t>
         </is>
       </c>
     </row>
@@ -510,7 +510,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Unchanged from the original export</t>
+          <t>Unchanged</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Unchanged from the original export</t>
+          <t>Unchanged</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Unchanged from the original export</t>
+          <t>Unchanged</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB242"/>
+  <dimension ref="A1:AB246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1160,12 +1160,14 @@
           <t>Syrian former employees</t>
         </is>
       </c>
-      <c r="AA5" t="n">
-        <v>0</v>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>ECCHR — Lafarge Case: https://www.ecchr.eu/en/case/lafarge-in-syria/ | SJAC — Corporate Accountability: https://syriaaccountability.org/ | UJAR 2025: https://trialinternational.org/universal-jurisdiction-tools/universal-jurisdiction-annual-review-ujar/ | Amnesty France — Compétence universelle: https://competenceuniverselle.amnesty.fr/ | Sherpa — Lafarge Dossier: https://www.asso-sherpa.org/lafarge</t>
+          <t>ECCHR — Lafarge Case: https://www.ecchr.eu/en/case/lafarge-in-syria/ | SJAC — Corporate Accountability: https://syriaaccountability.org/ | UJAR 2025: https://trialinternational.org/universal-jurisdiction-tools/universal-jurisdiction-annual-review-ujar/ | Amnesty France — Compétence universelle: https://competenceuniverselle.amnesty.fr/ | Sherpa — Lafarge Dossier: https://www.asso-sherpa.org/lafarge; BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/</t>
         </is>
       </c>
     </row>
@@ -2101,6 +2103,11 @@
           <t>1</t>
         </is>
       </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2804,6 +2811,11 @@
           <t>1</t>
         </is>
       </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4080,6 +4092,11 @@
       <c r="AA35" t="n">
         <v>0</v>
       </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4173,6 +4190,11 @@
       <c r="AA36" t="n">
         <v>0</v>
       </c>
+      <c r="AB36" t="inlineStr">
+        <is>
+          <t>BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4266,6 +4288,11 @@
       <c r="AA37" t="n">
         <v>0</v>
       </c>
+      <c r="AB37" t="inlineStr">
+        <is>
+          <t>BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6035,6 +6062,11 @@
       <c r="AA55" t="n">
         <v>0</v>
       </c>
+      <c r="AB55" t="inlineStr">
+        <is>
+          <t>BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -9372,7 +9404,7 @@
       </c>
       <c r="AB89" t="inlineStr">
         <is>
-          <t>CPCR — Collectif des parties civiles pour le Rwanda (chroniques d audience, arrêts, lettres de motivation): https://www.collectifpartiescivilesrwanda.fr/proces/ | Amnesty France — Compétence universelle: https://competenceuniverselle.amnesty.fr/</t>
+          <t>CPCR — Collectif des parties civiles pour le Rwanda (chroniques d audience, arrêts, lettres de motivation): https://www.collectifpartiescivilesrwanda.fr/proces/ | Amnesty France — Compétence universelle: https://competenceuniverselle.amnesty.fr/; BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/</t>
         </is>
       </c>
     </row>
@@ -9468,6 +9500,11 @@
       <c r="AA90" t="n">
         <v>0</v>
       </c>
+      <c r="AB90" t="inlineStr">
+        <is>
+          <t>BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -11020,6 +11057,11 @@
       <c r="AA106" t="n">
         <v>0</v>
       </c>
+      <c r="AB106" t="inlineStr">
+        <is>
+          <t>BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -11221,6 +11263,11 @@
       <c r="AA108" t="n">
         <v>0</v>
       </c>
+      <c r="AB108" t="inlineStr">
+        <is>
+          <t>BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -11899,6 +11946,11 @@
       <c r="AA115" t="n">
         <v>0</v>
       </c>
+      <c r="AB115" t="inlineStr">
+        <is>
+          <t>BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -18130,7 +18182,7 @@
       </c>
       <c r="AB178" t="inlineStr">
         <is>
-          <t>Amnesty France — Cartographie compétence universelle: https://competenceuniverselle.amnesty.fr/affaire/qosmos/ | FIDH — Qosmos / Syrie: https://www.fidh.org/fr/themes/mondialisation-droits-humains/</t>
+          <t>Amnesty France — Cartographie compétence universelle: https://competenceuniverselle.amnesty.fr/affaire/qosmos/ | FIDH — Qosmos / Syrie: https://www.fidh.org/fr/themes/mondialisation-droits-humains/; BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/</t>
         </is>
       </c>
     </row>
@@ -19173,6 +19225,11 @@
       <c r="AA188" t="n">
         <v>2</v>
       </c>
+      <c r="AB188" t="inlineStr">
+        <is>
+          <t>BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -21942,7 +21999,7 @@
       </c>
       <c r="AB216" t="inlineStr">
         <is>
-          <t>Added from the 2026-07 Legal Data Hunter enrichment (see enrichment/ folder)</t>
+          <t>Added from the 2026-07 Legal Data Hunter enrichment (see enrichment/ folder); BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/</t>
         </is>
       </c>
     </row>
@@ -22042,7 +22099,7 @@
       </c>
       <c r="AB217" t="inlineStr">
         <is>
-          <t>Added from the 2026-07 Legal Data Hunter enrichment (see enrichment/ folder)</t>
+          <t>Added from the 2026-07 Legal Data Hunter enrichment (see enrichment/ folder); BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/</t>
         </is>
       </c>
     </row>
@@ -24458,6 +24515,406 @@
       <c r="AB242" t="inlineStr">
         <is>
           <t>Referenced in Bryce/Johns/Langer, LJIL 2025 (doi:10.1017/S0922156524000244) and/or Langer &amp; Eason, EJIL 2019 (doi:10.1093/ejil/chz050); details to be re-verified against primary sources.</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>us-doe-unocal</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Doe v. Unocal (US — Myanmar, Yadana pipeline forced labour)</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>395 F.3d 932</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>U.S. Court of Appeals, Ninth Circuit</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>2002-09-18</t>
+        </is>
+      </c>
+      <c r="G243" t="n">
+        <v>2002</v>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>Myanmar</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>Forced labour; Murder; Rape (civil, corporate defendant)</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>Alien Tort Statute / TVPA (civil)</t>
+        </is>
+      </c>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>civil</t>
+        </is>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>Claims reinstated (2002); settled for compensation (2005)</t>
+        </is>
+      </c>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>civil_litigation</t>
+        </is>
+      </c>
+      <c r="N243" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O243" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="Q243" t="inlineStr">
+        <is>
+          <t>Burmese villagers sued Unocal over forced labour, killings and rape by the Myanmar military securing the Yadana gas pipeline. The Ninth Circuit held that aiding and abetting forced labour is actionable under the ATS — the first corporate atrocity case to head towards trial before its 2005 settlement, the founding precedent of corporate ATS litigation.</t>
+        </is>
+      </c>
+      <c r="R243" t="inlineStr">
+        <is>
+          <t>Forced labour as a modern variant of slavery requiring no state action; corporate aiding-and-abetting liability (knowing practical assistance standard).</t>
+        </is>
+      </c>
+      <c r="S243" t="inlineStr">
+        <is>
+          <t>https://www.courtlistener.com/opinion/789011/john-doe-i-individually-as-administrator-of-the-estate-of-his-deceased/</t>
+        </is>
+      </c>
+      <c r="AA243" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB243" t="inlineStr">
+        <is>
+          <t>BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/ — added from the 2026-07 Legal Data Hunter enrichment (batch 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>us-talisman-sudan</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Presbyterian Church of Sudan v. Talisman Energy (US — Sudan oil)</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>582 F.3d 244</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>U.S. Court of Appeals, Second Circuit</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>2009-10-02</t>
+        </is>
+      </c>
+      <c r="G244" t="n">
+        <v>2009</v>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>Sudan</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>Genocide; Crimes against humanity; War crimes (aiding and abetting — civil, corporate defendant)</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>Alien Tort Statute / TVPA (civil)</t>
+        </is>
+      </c>
+      <c r="K244" t="inlineStr">
+        <is>
+          <t>civil</t>
+        </is>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>Dismissed (purpose standard not met); cert denied (2010)</t>
+        </is>
+      </c>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>civil_litigation</t>
+        </is>
+      </c>
+      <c r="N244" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O244" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="Q244" t="inlineStr">
+        <is>
+          <t>Sudanese plaintiffs alleged Talisman Energy assisted the Sudanese government’s ethnic-cleansing campaign around its oil concessions. The Second Circuit affirmed dismissal, holding that ATS aiding-and-abetting liability requires acting with the PURPOSE of facilitating the crimes, not mere knowledge — the restrictive mens rea pole of the corporate-complicity debate.</t>
+        </is>
+      </c>
+      <c r="R244" t="inlineStr">
+        <is>
+          <t>Purpose (not knowledge) standard for aiding-and-abetting under the ATS, drawn from customary international law.</t>
+        </is>
+      </c>
+      <c r="S244" t="inlineStr">
+        <is>
+          <t>https://www.courtlistener.com/opinion/2287736/presbyterian-church-of-sudan-v-talisman-energy-inc/</t>
+        </is>
+      </c>
+      <c r="AA244" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB244" t="inlineStr">
+        <is>
+          <t>BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/ — added from the 2026-07 Legal Data Hunter enrichment (batch 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>us-nestle-doe</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Doe v. Nestlé / Cargill (US — Côte d’Ivoire child slavery)</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>593 U.S. 628 (2021)</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Supreme Court of the United States / Ninth Circuit</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>2021-06-17</t>
+        </is>
+      </c>
+      <c r="G245" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>Côte d’Ivoire</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>Child slavery; Forced labour (aiding and abetting — civil, corporate defendants)</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>Alien Tort Statute / TVPA (civil)</t>
+        </is>
+      </c>
+      <c r="K245" t="inlineStr">
+        <is>
+          <t>civil</t>
+        </is>
+      </c>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>Dismissed by the Supreme Court (extraterritoriality); litigation continued on other grounds</t>
+        </is>
+      </c>
+      <c r="M245" t="inlineStr">
+        <is>
+          <t>civil_litigation</t>
+        </is>
+      </c>
+      <c r="N245" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O245" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="Q245" t="inlineStr">
+        <is>
+          <t>Former child slaves on Ivorian cocoa farms sued Nestlé USA and Cargill for aiding and abetting child slavery through purchasing and technical support. After two decades and three Ninth Circuit opinions, the Supreme Court held that general corporate activity in the United States is insufficient to displace the presumption against extraterritoriality — with Jesner v. Arab Bank (584 U.S. 241 (2018), barring ATS suits against foreign corporations), the case that closed most of the corporate ATS route.</t>
+        </is>
+      </c>
+      <c r="R245" t="inlineStr">
+        <is>
+          <t>Domestic-conduct requirement post-Kiobel applied to corporate defendants; aiding-and-abetting pleading standards (9th Cir. 2018).</t>
+        </is>
+      </c>
+      <c r="S245" t="inlineStr">
+        <is>
+          <t>https://www.courtlistener.com/opinion/4892569/nestle-usa-inc-v-doe/</t>
+        </is>
+      </c>
+      <c r="AA245" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB245" t="inlineStr">
+        <is>
+          <t>BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/ — added from the 2026-07 Legal Data Hunter enrichment (batch 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>us-chiquita-mdl</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>In re Chiquita Brands (US — Colombia, AUC financing)</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>MDL No. 08-md-01916 (S.D. Fla.)</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>U.S. District Court, Southern District of Florida</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>2024-06-10</t>
+        </is>
+      </c>
+      <c r="G246" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>Torture; Extrajudicial killing; Crimes against humanity (financing paramilitaries — civil, corporate defendant)</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>Alien Tort Statute / TVPA (civil)</t>
+        </is>
+      </c>
+      <c r="K246" t="inlineStr">
+        <is>
+          <t>civil</t>
+        </is>
+      </c>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t>June 2024: first US jury verdict holding a corporation liable for financing paramilitary abuses ($38.3M); earlier 2007 DOJ guilty plea ($25M fine)</t>
+        </is>
+      </c>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>civil_litigation</t>
+        </is>
+      </c>
+      <c r="N246" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O246" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="Q246" t="inlineStr">
+        <is>
+          <t>Thousands of Colombian victims sued Chiquita over its payments of about $1.7 million to the AUC paramilitaries (2001-2004), to which Chiquita had pleaded guilty in the 2007 US criminal case. After seventeen years of MDL litigation, a federal jury in June 2024 found Chiquita liable for eight AUC murders — the first time a US jury held an American corporation liable for financing human rights abuses abroad.</t>
+        </is>
+      </c>
+      <c r="R246" t="inlineStr">
+        <is>
+          <t>Corporate civil liability for financing a designated terrorist/paramilitary organisation; TVPA and Colombian-law claims surviving Kiobel.</t>
+        </is>
+      </c>
+      <c r="S246" t="inlineStr">
+        <is>
+          <t>https://www.courtlistener.com/opinion/2112999/in-re-chiquita-brands-international-inc/</t>
+        </is>
+      </c>
+      <c r="AA246" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB246" t="inlineStr">
+        <is>
+          <t>BHRRC Corporate Legal Accountability: https://www.business-humanrights.org/en/big-issues/corporate-legal-accountability/case-profiles/ — added from the 2026-07 Legal Data Hunter enrichment (batch 7)</t>
         </is>
       </c>
     </row>
@@ -24472,7 +24929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L211"/>
+  <dimension ref="A1:L223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34424,6 +34881,586 @@
       <c r="J211" t="inlineStr">
         <is>
           <t>5 years; died pending appeal, so never final — but the doctrinal foundation of the modern German NS-accessory line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>lafarge-syria</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Lafarge S.A.</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>2021-09-07</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Cour de cassation — corporate complicity in crimes against humanity</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Cour de cassation, Chambre criminelle</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>supreme_court</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>Pourvois n° 19-87.367, 19-87.376, 19-87.662 (FS-B)</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>https://www.courdecassation.fr/decision/6137092ff585960512dfe635</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>French</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>Landmark joined arrêt: knowingly paying several million dollars to an organisation whose object is exclusively criminal suffices to characterise complicity in crimes against humanity, regardless of the pursuit of a commercial activity. Sibling arrêts of the same day: n° 19-87.031, 19-87.036 (endangerment of employees), 19-87.040.</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>us-doe-unocal</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr"/>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>2000-08-31</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>District court — summary judgment for defendants</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>U.S. District Court, C.D. California</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>first_instance</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>110 F. Supp. 2d 1294 (C.D. Cal. 2000)</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>https://www.courtlistener.com/opinion/2568578/doe-i-v-unocal-corp/</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>Summary judgment order later reversed in relevant part by the Ninth Circuit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>us-doe-unocal</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr"/>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>2002-09-18</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Ninth Circuit — aiding and abetting forced labour actionable</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>U.S. Court of Appeals, Ninth Circuit</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>appeal</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>395 F.3d 932 (9th Cir. 2002)</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>https://www.courtlistener.com/opinion/789011/john-doe-i-individually-as-administrator-of-the-estate-of-his-deceased/</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>Panel opinion (395 F.3d 932); en banc rehearing granted, case settled in 2005 before decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>us-talisman-sudan</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr"/>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>2003-03-19</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>District court — motion to dismiss largely denied</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>U.S. District Court, S.D. New York</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>first_instance</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>244 F. Supp. 2d 289 (S.D.N.Y. 2003)</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>https://www.courtlistener.com/opinion/2287736/presbyterian-church-of-sudan-v-talisman-energy-inc/</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>Early ruling allowing genocide/CAH aiding-and-abetting claims to proceed (244 F. Supp. 2d 289).</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>us-talisman-sudan</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr"/>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>2006-09-12</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>District court — summary judgment for Talisman</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>U.S. District Court, S.D. New York</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>first_instance</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>453 F. Supp. 2d 633 (S.D.N.Y. 2006)</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>https://www.courtlistener.com/opinion/2475432/presbyterian-church-of-sudan-v-talisman-energy/</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>Summary judgment; affirmed by the Second Circuit (582 F.3d 244, 2 Oct 2009 — purpose standard).</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>us-talisman-sudan</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr"/>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>2010-10-04</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Supreme Court — certiorari denied</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Supreme Court of the United States</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>supreme_court</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>562 U.S. 946 (2010)</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>https://www.courtlistener.com/opinion/7339192/presbyterian-church-of-sudan-v-talisman-energy-inc/</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>Cert denied, leaving the Second Circuit purpose standard in place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>us-nestle-doe</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr"/>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>2014-09-04</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Ninth Circuit — claims reinstated</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>U.S. Court of Appeals, Ninth Circuit</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>appeal</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>No. 10-56739</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>https://www.courtlistener.com/opinion/3066204/john-doe-i-v-nestle-usa/</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>766 F.3d 1013 / 738 F.3d 1048 line: corporate liability under the ATS survives Kiobel at the pleading stage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>us-nestle-doe</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr"/>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>2018-10-23</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Ninth Circuit — amended complaint allowed</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>U.S. Court of Appeals, Ninth Circuit</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>appeal</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>No. 17-55435</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>https://www.courtlistener.com/opinion/4546316/john-doe-v-nestle-sa/</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>906 F.3d 1120: domestic conduct (funding and supply decisions from the US) sufficiently alleged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>us-nestle-doe</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr"/>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>2021-06-17</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Supreme Court — Nestlé USA, Inc. v. Doe</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Supreme Court of the United States</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>supreme_court</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>593 U.S. 628 (2021)</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>https://www.courtlistener.com/opinion/4892569/nestle-usa-inc-v-doe/</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>General corporate activity in the US cannot establish the domestic application of the ATS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>us-chiquita-mdl</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr"/>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>2011-06-03</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>MDL — motions to dismiss largely denied</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>U.S. District Court, S.D. Florida (Marra, J.)</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>first_instance</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>08-md-01916-KAM</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>https://www.courtlistener.com/opinion/2112999/in-re-chiquita-brands-international-inc/</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>792 F. Supp. 2d 1301: TVPA and ATS claims over AUC financing proceed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>us-chiquita-mdl</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr"/>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>2016-06-01</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>MDL — rulings on claims against individual executives</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>U.S. District Court, S.D. Florida (Marra, J.)</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>first_instance</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>08-md-01916-KAM</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>https://www.courtlistener.com/opinion/7320659/in-re-chiquita-brands-international-inc/</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>Motions to dismiss the claims against former Chiquita executives granted in part and denied in part.</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>us-chiquita-mdl</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr"/>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>2018-01-03</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>MDL — New Tribes Mission claims ruling</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>U.S. District Court, S.D. Florida (Marra, J.)</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>first_instance</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>08-md-01916-KAM</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>https://www.courtlistener.com/opinion/7327957/in-re-chiquita-brands-intl-inc/</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>Ruling in the action over the murders of six US citizens by the FARC/AUC context.</t>
         </is>
       </c>
     </row>

</xml_diff>